<commit_message>
fix: remove fixed column widths in minnano cache Co-authored-by: monkeycode-ai <monkeycode-ai@chaitin.com>
</commit_message>
<xml_diff>
--- a/resources/userdata/minnano_cache.xlsx
+++ b/resources/userdata/minnano_cache.xlsx
@@ -426,22 +426,6 @@
   </sheetPr>
   <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="6" customWidth="1" min="4" max="4"/>
-    <col width="6" customWidth="1" min="5" max="5"/>
-    <col width="6" customWidth="1" min="6" max="6"/>
-    <col width="6" customWidth="1" min="7" max="7"/>
-    <col width="6" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="10" customWidth="1" min="11" max="11"/>
-    <col width="10" customWidth="1" min="12" max="12"/>
-    <col width="200" customWidth="1" min="13" max="13"/>
-    <col width="45" customWidth="1" min="14" max="14"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">

</xml_diff>

<commit_message>
feat: add roman name column to minnano cache Co-authored-by: monkeycode-ai <monkeycode-ai@chaitin.com>
</commit_message>
<xml_diff>
--- a/resources/userdata/minnano_cache.xlsx
+++ b/resources/userdata/minnano_cache.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O1"/>
+  <dimension ref="A1:P1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -495,10 +495,15 @@
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
+          <t>罗马音</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
           <t>维基百科简介</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>minnano url</t>
         </is>

</xml_diff>

<commit_message>
chore: remove roman name column and jp_name/en_name parsing Co-authored-by: monkeycode-ai <monkeycode-ai@chaitin.com>
</commit_message>
<xml_diff>
--- a/resources/userdata/minnano_cache.xlsx
+++ b/resources/userdata/minnano_cache.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P1"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -495,15 +495,10 @@
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>罗马音</t>
+          <t>维基百科简介</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>维基百科简介</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>minnano url</t>
         </is>

</xml_diff>